<commit_message>
final/ refreshed from live + ArmSoft import for batch 2026-10-14-siruk
Source of truth, barcodes and the 303 per-kg sheets re-read from the live
catalogue: 40 new variants (23 Felix / Pro Plan + 17 added 2026-10-13),
5 barcodes, 4 per-kg prices. ArmSoft: 22 new goods 1474-1495 (new-goods.xml
+ prices.xlsx), Pro Plan loose PLU 00106; target XML and code map in step.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/final/Siruk-hx-303-prices-cat.xlsx
+++ b/final/Siruk-hx-303-prices-cat.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>4150</v>
+        <v>4350</v>
       </c>
     </row>
     <row r="23">
@@ -1056,6 +1056,26 @@
       </c>
       <c r="D32" t="n">
         <v>6000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Կեր կատուների Pro Plan Sterilised Adult Renal Plus, հնդկահավ, 10 կգ</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Pro Plan Sterilised Adult Renal Plus — Turkey 10 kg</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>00106</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>3950</v>
       </c>
     </row>
   </sheetData>

</xml_diff>